<commit_message>
testing 50 test cases
</commit_message>
<xml_diff>
--- a/It23578500_Assignment_1_Test_Cases_.xlsx
+++ b/It23578500_Assignment_1_Test_Cases_.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dewmini Iddamalgoda\Desktop\test_automation123\test_automation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/09a55667ea5cd5a1/Pictures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66F7F156-96C1-4DBF-AAE3-1490AEE9B251}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="69" documentId="11_F04DF6EBDF7605FDEA5B22D431EE2AD5AB368FAD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56646177-D219-47A4-8CFD-BBD13E431AA1}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test cases" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="289">
   <si>
     <t>TC ID</t>
   </si>
@@ -59,6 +59,12 @@
     <t>ඔයාලා අද එනවාද?</t>
   </si>
   <si>
+    <t>ඔයාලා අද එනවද?</t>
+  </si>
+  <si>
+    <t>FAIL</t>
+  </si>
+  <si>
     <t>Question forms</t>
   </si>
   <si>
@@ -74,6 +80,9 @@
     <t>ඔයා කවුරු එක්කද ගියේ?</t>
   </si>
   <si>
+    <t>ඔය කව්රු එක්කද ගියේ?</t>
+  </si>
+  <si>
     <t>Rationale: The word “giye?” shows a question form.</t>
   </si>
   <si>
@@ -83,12 +92,15 @@
     <t>M</t>
   </si>
   <si>
-    <t>Malli, danma gedarata enna kiyanna.</t>
+    <t>Malli, danma gedarata ena kiyanna.</t>
   </si>
   <si>
     <t>මල්ලි, දැන්ම ගෙදරට එන්න කියන්න.</t>
   </si>
   <si>
+    <t>මල්ලි, දැන්ම ගෙදරට එන කියන්න.</t>
+  </si>
+  <si>
     <t>Command forms</t>
   </si>
   <si>
@@ -98,9 +110,6 @@
     <t>Neg_0004</t>
   </si>
   <si>
-    <t>Me file eka ikmanata upload karanna.</t>
-  </si>
-  <si>
     <t>මේ file එක ඉක්මනට upload කරන්න.</t>
   </si>
   <si>
@@ -110,12 +119,15 @@
     <t>Neg_0005</t>
   </si>
   <si>
-    <t>suba dawask wewa!</t>
+    <t>suba dawask weewa!</t>
   </si>
   <si>
     <t>සුබ දවසක් වේවා!</t>
   </si>
   <si>
+    <t>සුබ දවසක් වීවා!</t>
+  </si>
+  <si>
     <t>Greetings</t>
   </si>
   <si>
@@ -125,24 +137,21 @@
     <t>Neg_0006</t>
   </si>
   <si>
-    <t>Oyalata suba pathum aluth gamanakata!</t>
+    <t>Oyalta suba pathum aluth gamanakata!</t>
   </si>
   <si>
     <t>ඔයාලට සුබ පැතුම් අලුත් ගමනකට!</t>
   </si>
   <si>
+    <t>ඔයාලාට සුබ පැතුම් අලුත් ගමනකට!</t>
+  </si>
+  <si>
     <t>Rationale: “suba pathum” is a greeting/congratulatory phrase.</t>
   </si>
   <si>
     <t>Neg_0007</t>
   </si>
   <si>
-    <t>mata podi udawwak karanna puluwanda?</t>
-  </si>
-  <si>
-    <t>මට පොඩි උදව්වක් කරන්න පුළුවන්ද?</t>
-  </si>
-  <si>
     <t>Requests</t>
   </si>
   <si>
@@ -152,24 +161,12 @@
     <t>Neg_0008</t>
   </si>
   <si>
-    <t>oyata welawak thiyenawanam mata call karanna.</t>
-  </si>
-  <si>
-    <t>ඔයාට වෙලාවක් තියෙනවානම් මට call කරන්න.</t>
-  </si>
-  <si>
     <t>Rationale: “welawak thiyenawanam” makes it a polite request.</t>
   </si>
   <si>
     <t>Neg_0009</t>
   </si>
   <si>
-    <t>hari hari, api balamu.</t>
-  </si>
-  <si>
-    <t>හරි හරි, අපි බලමු.</t>
-  </si>
-  <si>
     <t>Repeated words</t>
   </si>
   <si>
@@ -179,24 +176,30 @@
     <t>Neg_0010</t>
   </si>
   <si>
-    <t>yamu yamu, parakku wenawa.</t>
+    <t>ymu ymu, prkku wenawa.</t>
   </si>
   <si>
     <t>යමු යමු, පරක්කු වෙනවා.</t>
   </si>
   <si>
+    <t>යමු යමු, පර්ක්කු වෙනවා.</t>
+  </si>
+  <si>
     <t>Evidence: “yamu yamu” repeats the same word.</t>
   </si>
   <si>
     <t>Neg_0011</t>
   </si>
   <si>
-    <t>mama enawa... oyala innawada?</t>
+    <t>mama enawa... oyala innavada?</t>
   </si>
   <si>
     <t>මම එනවා... ඔයාලා ඉන්නවාද?</t>
   </si>
   <si>
+    <t>මම එනවා... ඔයාලා ඉන්නවද?</t>
+  </si>
+  <si>
     <t>Inputs with punctuation marks</t>
   </si>
   <si>
@@ -206,24 +209,30 @@
     <t>Neg_0012</t>
   </si>
   <si>
-    <t>ane, eka denna! mata one.</t>
+    <t>ane, eka denna! mata oni.</t>
   </si>
   <si>
     <t>අනේ, ඒක දෙන්න! මට ඕනේ.</t>
   </si>
   <si>
+    <t>අනේ, එක දෙන්න! මට ඕනි.</t>
+  </si>
+  <si>
     <t>Evidence: Uses comma, exclamation mark, and full stop.</t>
   </si>
   <si>
     <t>Neg_0013</t>
   </si>
   <si>
-    <t>mn heta clz ekata ennam.</t>
+    <t>mn heta clz ekata ennm.</t>
   </si>
   <si>
     <t>මං හෙට class එකට එන්නම්.</t>
   </si>
   <si>
+    <t>මන් හෙට class එකට එන්නම්.</t>
+  </si>
+  <si>
     <t>Romanization / Spelling variants</t>
   </si>
   <si>
@@ -233,24 +242,30 @@
     <t>Neg_0014</t>
   </si>
   <si>
-    <t>oyta mage msg eka labunada?</t>
+    <t>oyta mage msg eka labunda?</t>
   </si>
   <si>
     <t>ඔයාට මගේ message එක ලැබුණාද?</t>
   </si>
   <si>
+    <t>ඔයාට මගේ msg එක ලැබුන්ද?</t>
+  </si>
+  <si>
     <t>Evidence: “oyta” is a shortened variant of “oyata”; “msg” is a spelling variant of message.</t>
   </si>
   <si>
     <t>Neg_0015</t>
   </si>
   <si>
-    <t>mama dan lunch ganna yanne.</t>
+    <t>mama dan lunch ganna yane.</t>
   </si>
   <si>
     <t>මම දැන් lunch ගන්න යන්නේ.</t>
   </si>
   <si>
+    <t>මම දැන් lunch ගන්න යනේ.</t>
+  </si>
+  <si>
     <t>Isolated English word insertions</t>
   </si>
   <si>
@@ -260,24 +275,12 @@
     <t>Neg_0016</t>
   </si>
   <si>
-    <t>ape team eka heta enawa.</t>
-  </si>
-  <si>
-    <t>අපේ team එක හෙට එනවා.</t>
-  </si>
-  <si>
     <t>Evidence: Single English word “team” is embedded.</t>
   </si>
   <si>
     <t>Neg_0017</t>
   </si>
   <si>
-    <t>eya ada work from home karanawa.</t>
-  </si>
-  <si>
-    <t>එයා අද work from home කරනවා.</t>
-  </si>
-  <si>
     <t>Multi-word English phrases</t>
   </si>
   <si>
@@ -287,19 +290,25 @@
     <t>Neg_0018</t>
   </si>
   <si>
-    <t>api dan on the way, ikmanata ennam.</t>
+    <t>api dan on da way, ikmanta ennm.</t>
   </si>
   <si>
     <t>අපි දැන් on the way, ඉක්මනට එන්නම්.</t>
   </si>
   <si>
+    <t>අපි දැන් ඔන් ද වය්, ඉක්මනට එන්නම්.</t>
+  </si>
+  <si>
     <t>Evidence: “on the way” is a multi-word English phrase.</t>
   </si>
   <si>
     <t>Neg_0019</t>
   </si>
   <si>
-    <t>oyage email eka mata ewanna.</t>
+    <t>oyage e-mail eka mata ewnna.</t>
+  </si>
+  <si>
+    <t>ඔයාගේ e-mail එක මට එවන්න.</t>
   </si>
   <si>
     <t>ඔයාගේ email එක මට එවන්න.</t>
@@ -314,24 +323,30 @@
     <t>Neg_0020</t>
   </si>
   <si>
-    <t>phone eke bluetooth on karanna.</t>
+    <t>phone eke bluethooth on karanna.</t>
   </si>
   <si>
     <t>phone එකේ bluetooth on කරන්න.</t>
   </si>
   <si>
+    <t>phone එකේ bluethooth on කරන්න.</t>
+  </si>
+  <si>
     <t>Evidence: “bluetooth” and “on” are digital/technology terms.</t>
   </si>
   <si>
     <t>Neg_0021</t>
   </si>
   <si>
-    <t>ape group eka Telegram eke thiyenne.</t>
+    <t>ape grp eka Telegram eke thiyenne.</t>
   </si>
   <si>
     <t>අපේ group එක Telegram එකේ තියෙන්නේ.</t>
   </si>
   <si>
+    <t>අපේ grp එක Telegram එකේ තියෙන්නේ.</t>
+  </si>
+  <si>
     <t>Platform/App names</t>
   </si>
   <si>
@@ -341,9 +356,6 @@
     <t>Neg_0022</t>
   </si>
   <si>
-    <t>mata Google Meet link eka ewanna.</t>
-  </si>
-  <si>
     <t>මට Google Meet link එක එවන්න.</t>
   </si>
   <si>
@@ -359,6 +371,9 @@
     <t>මගේ ID එක verify කරන්න.</t>
   </si>
   <si>
+    <t>මගේ ID ඒක verify කරන්න.</t>
+  </si>
+  <si>
     <t>English abbreviations/acronyms</t>
   </si>
   <si>
@@ -374,18 +389,24 @@
     <t>HR එකට මේක කියන්න ඕනේ.</t>
   </si>
   <si>
+    <t>HR ඒකට මේක කියන්න ඕනේ.</t>
+  </si>
+  <si>
     <t>Evidence: “HR” is an acronym.</t>
   </si>
   <si>
     <t>Neg_0025</t>
   </si>
   <si>
-    <t>mata lab eke practical ekak thiyenawa.</t>
+    <t>mata lab eke practical e kak thiyenawa.</t>
   </si>
   <si>
     <t>මට lab එකේ practical එකක් තියෙනවා.</t>
   </si>
   <si>
+    <t>මට lab එකේ practical ඒ කක් තියෙනවා.</t>
+  </si>
+  <si>
     <t>English clipped forms</t>
   </si>
   <si>
@@ -395,9 +416,6 @@
     <t>Neg_0026</t>
   </si>
   <si>
-    <t>heta maths exam eka thiyenawa.</t>
-  </si>
-  <si>
     <t>හෙට maths exam එක තියෙනවා.</t>
   </si>
   <si>
@@ -407,9 +425,6 @@
     <t>Neg_0027</t>
   </si>
   <si>
-    <t>api Kandy walata train eken yanawa.</t>
-  </si>
-  <si>
     <t>අපි Kandy වලට train එකෙන් යනවා.</t>
   </si>
   <si>
@@ -428,18 +443,24 @@
     <t>මම Colombo Fort එකේදී සෙට් වෙන්නම්.</t>
   </si>
   <si>
+    <t>මම Colombo Fort එකේදී set වෙන්නම්</t>
+  </si>
+  <si>
     <t>Evidence: “Colombo Fort” is a place name.</t>
   </si>
   <si>
     <t>Neg_0029</t>
   </si>
   <si>
-    <t>Nuwan ada office ekata awe naha.</t>
+    <t>Nuwan ada office ekata awe naa.</t>
   </si>
   <si>
     <t>නුවන් අද office එකට ආවේ නැහැ.</t>
   </si>
   <si>
+    <t>නුවන් අද office එකට ආවේ නෑ.</t>
+  </si>
+  <si>
     <t>Person names embedded</t>
   </si>
   <si>
@@ -449,21 +470,21 @@
     <t>Neg_0030</t>
   </si>
   <si>
-    <t>Kasuni mata potha dunna.</t>
+    <t>Kasuni mata pota dunna.</t>
   </si>
   <si>
     <t>කසුනි මට පොත දුන්නා.</t>
   </si>
   <si>
+    <t>කසුනි මට පොට දුන්නා.</t>
+  </si>
+  <si>
     <t>Evidence: “Kasuni” is a person name.</t>
   </si>
   <si>
     <t>Neg_0031</t>
   </si>
   <si>
-    <t>mata ticket 2k denna puluwanda?</t>
-  </si>
-  <si>
     <t>මට ticket 2ක් දෙන්න පුළුවන්ද?</t>
   </si>
   <si>
@@ -476,9 +497,6 @@
     <t>Neg_0032</t>
   </si>
   <si>
-    <t>api 3rd floor eke innawa.</t>
-  </si>
-  <si>
     <t>අපි 3rd floor එකේ ඉන්නවා.</t>
   </si>
   <si>
@@ -488,12 +506,6 @@
     <t>Neg_0033</t>
   </si>
   <si>
-    <t>mata LKR 1500k gewanna one.</t>
-  </si>
-  <si>
-    <t>මට LKR 1500ක් ගෙවන්න ඕනේ.</t>
-  </si>
-  <si>
     <t>Inputs with currency</t>
   </si>
   <si>
@@ -503,9 +515,6 @@
     <t>Neg_0034</t>
   </si>
   <si>
-    <t>USD 20k wage yanawa.</t>
-  </si>
-  <si>
     <t>USD 20ක් වගේ යනවා.</t>
   </si>
   <si>
@@ -515,12 +524,6 @@
     <t>Neg_0035</t>
   </si>
   <si>
-    <t>class eka 8.15am patan gannawa.</t>
-  </si>
-  <si>
-    <t>class එක 8.15am පටන් ගන්නවා.</t>
-  </si>
-  <si>
     <t>Inputs with time formats</t>
   </si>
   <si>
@@ -530,24 +533,21 @@
     <t>Neg_0036</t>
   </si>
   <si>
-    <t>api 6:45PM gedarin pitath wemu.</t>
+    <t>api 6:45PM gedarin pitat wemu.</t>
   </si>
   <si>
     <t>අපි 6:45PM ගෙදරින් පිටත් වෙමු.</t>
   </si>
   <si>
+    <t>අපි 6:45PM ගෙදරින් පිටත වෙමු.</t>
+  </si>
+  <si>
     <t>Evidence: “6:45PM” is a time format.</t>
   </si>
   <si>
     <t>Neg_0037</t>
   </si>
   <si>
-    <t>exam eka 2025-11-20ta thiyenawa.</t>
-  </si>
-  <si>
-    <t>exam එක 2025-11-20ට තියෙනවා.</t>
-  </si>
-  <si>
     <t>Inputs with dates</t>
   </si>
   <si>
@@ -557,24 +557,30 @@
     <t>Neg_0038</t>
   </si>
   <si>
-    <t>report ekata March 10 wenakan kal denna.</t>
+    <t>report ekata March 10 wenakam kal denna.</t>
   </si>
   <si>
     <t>report එකට March 10 වෙනකන් කල් දෙන්න.</t>
   </si>
   <si>
+    <t>report එකට March 10 වෙනකම් කල් දෙන්න.</t>
+  </si>
+  <si>
     <t>Evidence: “March 10” is a date reference.</t>
   </si>
   <si>
     <t>Neg_0039</t>
   </si>
   <si>
-    <t>mama 5km withara duwanawa.</t>
+    <t>man 5km withara duwanawa.</t>
   </si>
   <si>
     <t>මම 5km විතර දුවනවා.</t>
   </si>
   <si>
+    <t>මං 5km විතර දුවනවා.</t>
+  </si>
+  <si>
     <t>Inputs with unit of measurements</t>
   </si>
   <si>
@@ -584,12 +590,6 @@
     <t>Neg_0040</t>
   </si>
   <si>
-    <t>me table eka 2m diga athi.</t>
-  </si>
-  <si>
-    <t>මේ table එක 2m දිග ඇති.</t>
-  </si>
-  <si>
     <t>Evidence: “2m” is a measurement unit.</t>
   </si>
   <si>
@@ -602,6 +602,9 @@
     <t>මචං පට්ට වැඩක් කළේ උඹ.</t>
   </si>
   <si>
+    <t>මචං පට්ට වැඩක් කලේ උඹ.</t>
+  </si>
+  <si>
     <t>Slang and casual phrasing</t>
   </si>
   <si>
@@ -617,6 +620,9 @@
     <t>අඩෝ මේක නම් සුපිරි බං.</t>
   </si>
   <si>
+    <t>අඩො මේක නම් සුපිරි බන්.</t>
+  </si>
+  <si>
     <t>Evidence: “ado”, “supiri”, and “ban” are casual/slang words.</t>
   </si>
   <si>
@@ -629,6 +635,9 @@
     <t>මේ link එක open කරන්න: https://sliit.lk</t>
   </si>
   <si>
+    <t>මේ link එක open කරන්න: https://sliit.ල්ක්</t>
+  </si>
+  <si>
     <t>Online identifiers</t>
   </si>
   <si>
@@ -644,6 +653,9 @@
     <t>මට email එකක් එවන්න: testuser25@yahoo.com</t>
   </si>
   <si>
+    <t>මට email එකක් එවන්න: testuser25@yahoo.කොම්</t>
+  </si>
+  <si>
     <t>Evidence: Contains email address “testuser25@yahoo.com”.</t>
   </si>
   <si>
@@ -656,6 +668,9 @@
     <t>මම දැන් යනවා 😄</t>
   </si>
   <si>
+    <t>මම දැන් යනවා 😁</t>
+  </si>
+  <si>
     <t>Inputs containing emojis</t>
   </si>
   <si>
@@ -665,9 +680,6 @@
     <t>Neg_0046</t>
   </si>
   <si>
-    <t>oya hari hondai ❤️</t>
-  </si>
-  <si>
     <t>ඔයා හරි හොඳයි ❤️</t>
   </si>
   <si>
@@ -683,6 +695,9 @@
     <t>මට ඒ message එක කලින් ලැබුණා.</t>
   </si>
   <si>
+    <t>මට ඒ msg එක කලින් ලැබුණා.</t>
+  </si>
+  <si>
     <t>Evidence: “msg” is a chat-style spelling variant for message.</t>
   </si>
   <si>
@@ -695,6 +710,9 @@
     <t>මං ඔයාගේ number එක save කළා.</t>
   </si>
   <si>
+    <t>මන් ඔයාගේ නම් එක save කරා.</t>
+  </si>
+  <si>
     <t>Evidence: “mn” and “num” are shortened chat-style variants.</t>
   </si>
   <si>
@@ -707,6 +725,9 @@
     <t>මචං හෙට 4pm match එක බලන්න එනවාද?</t>
   </si>
   <si>
+    <t>මචන් හෙට 4pm match එක බලන්න එනවද?</t>
+  </si>
+  <si>
     <t>Question forms; Isolated English word insertions; Inputs with time formats; Slang and casual phrasing</t>
   </si>
   <si>
@@ -722,6 +743,9 @@
     <t>bro මට Rs. 500ක් online transfer කරන්න පුළුවන්ද?</t>
   </si>
   <si>
+    <t>bro මට Rs. 500ක් ඔන්ලයින් transfer කරන්න පුළුවන්ද?</t>
+  </si>
+  <si>
     <t>Requests; Inputs with currency; English digital terms; Slang and casual phrasing</t>
   </si>
   <si>
@@ -735,13 +759,142 @@
   </si>
   <si>
     <t>Length types: S = 30 characters or fewer, M = 31-299 characters, L = 300-450 characters.</t>
+  </si>
+  <si>
+    <t>Me file eka ikmnta uplod krnna plz.</t>
+  </si>
+  <si>
+    <t>මේ file එක ඉක්මනට upload කරන්න please.</t>
+  </si>
+  <si>
+    <t>mata podi udavvk karanna puluvanda pls ?</t>
+  </si>
+  <si>
+    <t>oyata welawak thiyenawanm mata call dnnko.</t>
+  </si>
+  <si>
+    <t>ඔයාට වෙලාවක් තියෙනවානම් මට call එකක් දෙන්නකෝ.</t>
+  </si>
+  <si>
+    <t>hari hariii, api balamuko.</t>
+  </si>
+  <si>
+    <t>හරි හරි, අපි බලමුකෝ.</t>
+  </si>
+  <si>
+    <t>ape teem ek heta enwada?</t>
+  </si>
+  <si>
+    <t>අපේ team එක හෙට එනවාද?</t>
+  </si>
+  <si>
+    <t>mata googlemeet link eka evnna.</t>
+  </si>
+  <si>
+    <t>api Kandywalata train eken yanawa.</t>
+  </si>
+  <si>
+    <t>mata LKR1K gevnna oni.</t>
+  </si>
+  <si>
+    <t>මට LKR 1K ගෙවන්න ඕනේ.</t>
+  </si>
+  <si>
+    <t>USD 20K wage yanva.</t>
+  </si>
+  <si>
+    <t>USD 20K වගේ යනවා.</t>
+  </si>
+  <si>
+    <t>class eka 8.15amta patan gannva.</t>
+  </si>
+  <si>
+    <t>class එක 8.15amට පටන් ගන්නවා.</t>
+  </si>
+  <si>
+    <t>exam eka 2025-11-20wenidawase thiyenva.</t>
+  </si>
+  <si>
+    <t>exam එක 2025-11-20 වෙනි දවසේ තියෙනවා.</t>
+  </si>
+  <si>
+    <t>me table aka 2mwage diga athi.</t>
+  </si>
+  <si>
+    <t>මේ table එක 2m වගේ දිග ඇති.</t>
+  </si>
+  <si>
+    <t>oyahri hondaai❤️</t>
+  </si>
+  <si>
+    <t>මට පොඩි උදව්වක් කරන්න පුළුවන්ද pls?</t>
+  </si>
+  <si>
+    <t>මට පොඩි උදව්වක් කරන්න පුළුවන්ද please ?</t>
+  </si>
+  <si>
+    <t>ඔයාට වෙලාවක් තියෙනවනම් මට call දාන්නකෝ.</t>
+  </si>
+  <si>
+    <t>හරි හරී, අපි බලමුකෝ.</t>
+  </si>
+  <si>
+    <t>අපේ ටීම් එක හෙට එනවද?</t>
+  </si>
+  <si>
+    <t>එයා අද Work From Home කරන්නේ.</t>
+  </si>
+  <si>
+    <t>eya adha Work From Home kernne.</t>
+  </si>
+  <si>
+    <t>එයා අද Work From Home කරන්න.</t>
+  </si>
+  <si>
+    <t>මට googlemeet link එක එවන්න.</t>
+  </si>
+  <si>
+    <t>heta mths exam eka thiyenawa.</t>
+  </si>
+  <si>
+    <t>හෙට මාත්ස් exam එක තියෙනවා.</t>
+  </si>
+  <si>
+    <t>අපි Kandywalaට train එකෙන් යනවා.</t>
+  </si>
+  <si>
+    <t>ඔයහරි හොඳයි❤️</t>
+  </si>
+  <si>
+    <t>මේ table එක 2mwage දිග ඇති.</t>
+  </si>
+  <si>
+    <t>exam එක 2025-11-20වෙනිදාවසේ තියෙනවා.</t>
+  </si>
+  <si>
+    <t>class එක 8.15මට පටන් ගන්නවා.</t>
+  </si>
+  <si>
+    <t>මට LKR 1ක් ගෙවන්න ඕනේ.</t>
+  </si>
+  <si>
+    <t>api 3rd floorek innva.</t>
+  </si>
+  <si>
+    <t>අපි 3rd floor එකක් ඉන්නවා.</t>
+  </si>
+  <si>
+    <t>mata ticket2 denna puluvnda?</t>
+  </si>
+  <si>
+    <t>මට ticket දෙන්න පුළුවන්ද?</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -761,6 +914,10 @@
       <sz val="11"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Times New Roman"/>
     </font>
   </fonts>
   <fills count="2">
@@ -783,7 +940,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -795,6 +952,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1014,219 +1174,259 @@
       <c r="D2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
+      <c r="E2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G2" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>9</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
+        <v>18</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G3" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="27.6" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
+        <v>24</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G4" s="4" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="27.6" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>25</v>
+        <v>246</v>
       </c>
       <c r="D5" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4" t="s">
-        <v>22</v>
-      </c>
       <c r="H5" s="4" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="4" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>9</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
+        <v>33</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G6" s="4" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="27.6" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D7" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4" t="s">
-        <v>31</v>
-      </c>
       <c r="H7" s="4" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="27.6" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>38</v>
+        <v>248</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
+        <v>268</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G8" s="4" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="27.6">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="27.6" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C9" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4" t="s">
-        <v>40</v>
-      </c>
       <c r="H9" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>9</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>47</v>
+        <v>251</v>
       </c>
       <c r="D10" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4" t="s">
+      <c r="H10" s="4" t="s">
         <v>49</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>9</v>
       </c>
       <c r="C11" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="E11" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
+      <c r="F11" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G11" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:8" ht="27.6" customHeight="1">
       <c r="A12" s="4" t="s">
         <v>55</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>56</v>
@@ -1234,580 +1434,688 @@
       <c r="D12" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
+      <c r="E12" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G12" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H12" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="27.6" customHeight="1">
+      <c r="A13" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G13" s="4" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="13" spans="1:8">
-      <c r="A13" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4" t="s">
-        <v>58</v>
-      </c>
       <c r="H13" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="27.6" customHeight="1">
       <c r="A14" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
+        <v>68</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G14" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="27.6" customHeight="1">
       <c r="A15" s="4" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C15" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="D15" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4" t="s">
-        <v>67</v>
-      </c>
       <c r="H15" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="27.6" customHeight="1">
       <c r="A16" s="4" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
+        <v>79</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G16" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="27.6" customHeight="1">
       <c r="A17" s="4" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>79</v>
+        <v>253</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
+        <v>254</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G17" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="27.6" customHeight="1">
       <c r="A18" s="4" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>83</v>
+        <v>274</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
+        <v>273</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G18" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H18" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="27.6" customHeight="1">
+      <c r="A19" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G19" s="4" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="19" spans="1:8">
-      <c r="A19" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4" t="s">
-        <v>85</v>
-      </c>
       <c r="H19" s="4" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="27.6" customHeight="1">
       <c r="A20" s="4" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
+        <v>95</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G20" s="4" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="27.6" customHeight="1">
       <c r="A21" s="4" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C21" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="D21" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4" t="s">
-        <v>94</v>
-      </c>
       <c r="H21" s="4" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="27.6" customHeight="1">
       <c r="A22" s="4" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
+        <v>106</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G22" s="4" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="27.6" customHeight="1">
       <c r="A23" s="4" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>106</v>
+        <v>255</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
+        <v>111</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G23" s="4" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="27.6" customHeight="1">
       <c r="A24" s="4" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="E24" s="4"/>
-      <c r="F24" s="4"/>
+        <v>115</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G24" s="4" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="27.6" customHeight="1">
       <c r="A25" s="4" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="E25" s="4"/>
-      <c r="F25" s="4"/>
+        <v>121</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G25" s="4" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="27.6" customHeight="1">
       <c r="A26" s="4" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4"/>
+        <v>126</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G26" s="4" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="27.6" customHeight="1">
       <c r="A27" s="4" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>124</v>
+        <v>277</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
+        <v>131</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G27" s="4" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="27.6" customHeight="1">
       <c r="A28" s="4" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>128</v>
+        <v>256</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
+        <v>134</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G28" s="4" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="27.6" customHeight="1">
       <c r="A29" s="4" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="E29" s="4"/>
-      <c r="F29" s="4"/>
+        <v>139</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G29" s="4" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="27.6" customHeight="1">
       <c r="A30" s="4" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="E30" s="4"/>
-      <c r="F30" s="4"/>
+        <v>144</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G30" s="4" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
     </row>
     <row r="31" spans="1:8">
       <c r="A31" s="4" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="E31" s="4"/>
-      <c r="F31" s="4"/>
+        <v>150</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G31" s="4" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="27.6" customHeight="1">
       <c r="A32" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>146</v>
+        <v>287</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="E32" s="4"/>
-      <c r="F32" s="4"/>
+        <v>154</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G32" s="4" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="27.6">
       <c r="A33" s="4" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>151</v>
+        <v>285</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="E33" s="4"/>
-      <c r="F33" s="4"/>
+        <v>158</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>286</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G33" s="4" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="27.6" customHeight="1">
       <c r="A34" s="4" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>155</v>
+        <v>257</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="E34" s="4"/>
-      <c r="F34" s="4"/>
+        <v>258</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G34" s="4" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
     </row>
     <row r="35" spans="1:8">
       <c r="A35" s="4" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>160</v>
+        <v>259</v>
       </c>
       <c r="D35" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G35" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="E35" s="4"/>
-      <c r="F35" s="4"/>
-      <c r="G35" s="4" t="s">
-        <v>157</v>
-      </c>
       <c r="H35" s="4" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="27.6" customHeight="1">
       <c r="A36" s="4" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>164</v>
+        <v>261</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="E36" s="4"/>
-      <c r="F36" s="4"/>
+        <v>262</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G36" s="4" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H36" s="4" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="27.6" customHeight="1">
+      <c r="A37" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G37" s="4" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="37" spans="1:8">
-      <c r="A37" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="D37" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="E37" s="4"/>
-      <c r="F37" s="4"/>
-      <c r="G37" s="4" t="s">
-        <v>166</v>
-      </c>
       <c r="H37" s="4" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="27.6" customHeight="1">
       <c r="A38" s="4" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>173</v>
+        <v>263</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="E38" s="4"/>
-      <c r="F38" s="4"/>
+        <v>264</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G38" s="4" t="s">
         <v>175</v>
       </c>
@@ -1815,12 +2123,12 @@
         <v>176</v>
       </c>
     </row>
-    <row r="39" spans="1:8">
+    <row r="39" spans="1:8" ht="27.6" customHeight="1">
       <c r="A39" s="4" t="s">
         <v>177</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>178</v>
@@ -1828,65 +2136,77 @@
       <c r="D39" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="E39" s="4"/>
-      <c r="F39" s="4"/>
+      <c r="E39" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G39" s="4" t="s">
         <v>175</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="40" spans="1:8">
       <c r="A40" s="4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="E40" s="4"/>
-      <c r="F40" s="4"/>
+        <v>184</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G40" s="4" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="27.6">
       <c r="A41" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G41" s="4" t="s">
         <v>186</v>
-      </c>
-      <c r="B41" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="D41" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="E41" s="4"/>
-      <c r="F41" s="4"/>
-      <c r="G41" s="4" t="s">
-        <v>184</v>
       </c>
       <c r="H41" s="4" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="42" spans="1:8">
+    <row r="42" spans="1:8" ht="27.6" customHeight="1">
       <c r="A42" s="4" t="s">
         <v>190</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>191</v>
@@ -1894,211 +2214,251 @@
       <c r="D42" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="E42" s="4"/>
-      <c r="F42" s="4"/>
+      <c r="E42" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G42" s="4" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="H42" s="4" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="27.6" customHeight="1">
+      <c r="A43" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G43" s="4" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="43" spans="1:8">
-      <c r="A43" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="B43" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C43" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="D43" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="E43" s="4"/>
-      <c r="F43" s="4"/>
-      <c r="G43" s="4" t="s">
-        <v>193</v>
-      </c>
       <c r="H43" s="4" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" ht="27.6" customHeight="1">
       <c r="A44" s="4" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="E44" s="4"/>
-      <c r="F44" s="4"/>
+        <v>203</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="F44" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G44" s="4" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8" ht="27.6">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" ht="27.6" customHeight="1">
       <c r="A45" s="4" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C45" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G45" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="D45" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="E45" s="4"/>
-      <c r="F45" s="4"/>
-      <c r="G45" s="4" t="s">
-        <v>202</v>
-      </c>
       <c r="H45" s="4" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
     </row>
     <row r="46" spans="1:8">
       <c r="A46" s="4" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="E46" s="4"/>
-      <c r="F46" s="4"/>
+        <v>214</v>
+      </c>
+      <c r="E46" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="F46" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G46" s="4" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="H46" s="4" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
     </row>
     <row r="47" spans="1:8">
       <c r="A47" s="4" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>214</v>
+        <v>267</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="E47" s="4"/>
-      <c r="F47" s="4"/>
+        <v>219</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G47" s="4" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="H47" s="4" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="27.6" customHeight="1">
       <c r="A48" s="4" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="E48" s="4"/>
-      <c r="F48" s="4"/>
+        <v>223</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G48" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" ht="27.6" customHeight="1">
       <c r="A49" s="4" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>223</v>
-      </c>
-      <c r="E49" s="4"/>
-      <c r="F49" s="4"/>
+        <v>228</v>
+      </c>
+      <c r="E49" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G49" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="H49" s="4" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="41.4" customHeight="1">
       <c r="A50" s="4" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="E50" s="4"/>
-      <c r="F50" s="4"/>
+        <v>233</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G50" s="4" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="H50" s="4" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="27.6" customHeight="1">
       <c r="A51" s="4" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>232</v>
-      </c>
-      <c r="E51" s="4"/>
-      <c r="F51" s="4"/>
+        <v>239</v>
+      </c>
+      <c r="E51" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="F51" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="G51" s="4" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="H51" s="4" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -2116,17 +2476,17 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="2" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="1" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="1" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
     </row>
   </sheetData>

</xml_diff>